<commit_message>
Remove ScreenSpot-excluded row from 3B comparison
</commit_message>
<xml_diff>
--- a/results/trace_3b_base_answer_annotation_combined.xlsx
+++ b/results/trace_3b_base_answer_annotation_combined.xlsx
@@ -11,8 +11,8 @@
     <sheet name="temp0.6" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'greedy'!$A$1:$N$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'temp0.6'!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'greedy'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'temp0.6'!$A$1:$N$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2094,52 +2094,8 @@
         <v>0.008780374689468075</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Average excl. ScreenSpot</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="6" t="n">
-        <v>35165</v>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="7" t="n">
-        <v>35.56110370370371</v>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>37.72743333333334</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>36.99430417458724</v>
-      </c>
-      <c r="I32" s="7" t="n">
-        <v>2.166329629629629</v>
-      </c>
-      <c r="J32" s="7" t="n">
-        <v>1.433200470883535</v>
-      </c>
-      <c r="K32" s="7" t="n">
-        <v>-0.7331291587460945</v>
-      </c>
-      <c r="L32" s="7" t="n">
-        <v>169.1511917876229</v>
-      </c>
-      <c r="M32" s="7" t="n">
-        <v>2297.851851851852</v>
-      </c>
-      <c r="N32" s="7" t="n">
-        <v>0.009383920142840251</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N32"/>
+  <autoFilter ref="A1:N31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2150,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3793,52 +3749,8 @@
         <v>0.001836419388906977</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Average excl. ScreenSpot</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="6" t="n">
-        <v>35165</v>
-      </c>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="7" t="n">
-        <v>33.75832222222222</v>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>36.9153</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>35.83877853295849</v>
-      </c>
-      <c r="I32" s="7" t="n">
-        <v>3.156977777777778</v>
-      </c>
-      <c r="J32" s="7" t="n">
-        <v>2.080456310736269</v>
-      </c>
-      <c r="K32" s="7" t="n">
-        <v>-1.07652146704151</v>
-      </c>
-      <c r="L32" s="7" t="n">
-        <v>131.4895156797896</v>
-      </c>
-      <c r="M32" s="7" t="n">
-        <v>1765.740740740741</v>
-      </c>
-      <c r="N32" s="7" t="n">
-        <v>0.001972450454751939</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N32"/>
+  <autoFilter ref="A1:N31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>